<commit_message>
chore: gitignore, dependances, brief et tracker a jour
</commit_message>
<xml_diff>
--- a/tracker-projet-tarification.xlsx
+++ b/tracker-projet-tarification.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ibrahimbello/Desktop/Projet tarification 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70FA2DE2-AC02-AB45-8A3B-C899F7D793CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A7F39C-B5D3-E740-BFDA-C99C0BA9D49F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14700" yWindow="1680" windowWidth="14720" windowHeight="16200" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17220" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de bord" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
   <si>
     <t>Moteur de tarification IARD  -  Tableau de bord</t>
   </si>
@@ -155,6 +155,30 @@
   </si>
   <si>
     <t xml:space="preserve">Explicabilite &amp; equite </t>
+  </si>
+  <si>
+    <t>Socle technique : repo, structure, venv, chargement donnees freMTPL2</t>
+  </si>
+  <si>
+    <t>Repo public en ligne (moteur-tarification-iard), structure projet, venv + requirements, script load_data reproductible, portefeuille 678013 polices charge en Parquet</t>
+  </si>
+  <si>
+    <t>Termine</t>
+  </si>
+  <si>
+    <t>EDA : integrite donnees, exposition, frequence, severite (queue epaisse)</t>
+  </si>
+  <si>
+    <t>Notebook EDA documente. Frequence 0.1007, offset justifie. Pas d'exces de zeros : ZIP ecarte. Severite : skewness 116.6, top 1% = 37.1% de la charge. BUG denominateur cout moyen : corriger via ClaimNbSev.</t>
+  </si>
+  <si>
+    <t>En cours</t>
+  </si>
+  <si>
+    <t>Correction denominateur (ClaimNbSev), notebook au propre, decomposition prime pure</t>
+  </si>
+  <si>
+    <t>Prime pure ref 167.11 EUR/annee-police. Frequence sur ClaimNb, severite sur ClaimNbSev, facteur correctif 0.732 a la recombinaison.</t>
   </si>
 </sst>
 </file>
@@ -294,7 +318,6 @@
   </cellStyleXfs>
   <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -351,6 +374,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -577,10 +601,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1000,10 +1024,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>3.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1450,68 +1474,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>46209</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="5">
         <f>'Suivi des phases'!E11</f>
-        <v>0</v>
+        <v>0.12727272727272726</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <f>'Suivi des phases'!C11</f>
         <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <f>'Suivi des phases'!F11</f>
-        <v>0</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <f>B6-B7</f>
-        <v>275</v>
+        <v>269.8</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="6">
         <f>COUNTIF('Suivi des phases'!D4:D10,"Termine")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1538,259 +1562,259 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="10">
         <v>15</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="12">
+      <c r="D4" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" s="11">
         <f t="shared" ref="E4:E10" si="0">IF(D4="Termine",1,IF(D4="En cours",0.5,0))</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="13">
+        <v>1</v>
+      </c>
+      <c r="F4" s="12">
         <f>SUMIF(Journal!$B$4:$B$203,A4,Journal!$D$4:$D$203)</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="14">
+        <v>2</v>
+      </c>
+      <c r="G4" s="13">
         <f>'Tableau de bord'!$B$3+H4*7</f>
         <v>46223</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="10">
         <v>40</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="16">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="F5" s="17">
+        <f>SUMIF(Journal!$B$4:$B$203,A5,Journal!$D$4:$D$203)</f>
+        <v>3.2</v>
+      </c>
+      <c r="G5" s="18">
+        <f>'Tableau de bord'!$B$3+H5*7</f>
+        <v>46251</v>
+      </c>
+      <c r="H5" s="10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="10">
+        <v>45</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="17">
+      <c r="E6" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F5" s="18">
-        <f>SUMIF(Journal!$B$4:$B$203,A5,Journal!$D$4:$D$203)</f>
+      <c r="F6" s="12">
+        <f>SUMIF(Journal!$B$4:$B$203,A6,Journal!$D$4:$D$203)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="19">
-        <f>'Tableau de bord'!$B$3+H5*7</f>
-        <v>46251</v>
-      </c>
-      <c r="H5" s="11">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="11">
+      <c r="G6" s="13">
+        <f>'Tableau de bord'!$B$3+H6*7</f>
+        <v>46279</v>
+      </c>
+      <c r="H6" s="10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="10">
         <v>45</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D7" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E7" s="16">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F6" s="13">
-        <f>SUMIF(Journal!$B$4:$B$203,A6,Journal!$D$4:$D$203)</f>
+      <c r="F7" s="17">
+        <f>SUMIF(Journal!$B$4:$B$203,A7,Journal!$D$4:$D$203)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="14">
-        <f>'Tableau de bord'!$B$3+H6*7</f>
-        <v>46279</v>
-      </c>
-      <c r="H6" s="11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="11">
+      <c r="G7" s="18">
+        <f>'Tableau de bord'!$B$3+H7*7</f>
+        <v>46307</v>
+      </c>
+      <c r="H7" s="10">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="10">
         <v>45</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D8" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="17">
+      <c r="E8" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F7" s="18">
-        <f>SUMIF(Journal!$B$4:$B$203,A7,Journal!$D$4:$D$203)</f>
+      <c r="F8" s="12">
+        <f>SUMIF(Journal!$B$4:$B$203,A8,Journal!$D$4:$D$203)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="19">
-        <f>'Tableau de bord'!$B$3+H7*7</f>
-        <v>46307</v>
-      </c>
-      <c r="H7" s="11">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="11">
+      <c r="G8" s="13">
+        <f>'Tableau de bord'!$B$3+H8*7</f>
+        <v>46335</v>
+      </c>
+      <c r="H8" s="10">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="10">
         <v>45</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D9" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E9" s="16">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F8" s="13">
-        <f>SUMIF(Journal!$B$4:$B$203,A8,Journal!$D$4:$D$203)</f>
+      <c r="F9" s="17">
+        <f>SUMIF(Journal!$B$4:$B$203,A9,Journal!$D$4:$D$203)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="14">
-        <f>'Tableau de bord'!$B$3+H8*7</f>
-        <v>46335</v>
-      </c>
-      <c r="H8" s="11">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="11">
-        <v>45</v>
-      </c>
-      <c r="D9" s="11" t="s">
+      <c r="G9" s="18">
+        <f>'Tableau de bord'!$B$3+H9*7</f>
+        <v>46363</v>
+      </c>
+      <c r="H9" s="10">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="10">
+        <v>40</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E10" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F9" s="18">
-        <f>SUMIF(Journal!$B$4:$B$203,A9,Journal!$D$4:$D$203)</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="19">
-        <f>'Tableau de bord'!$B$3+H9*7</f>
-        <v>46363</v>
-      </c>
-      <c r="H9" s="11">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="11">
-        <v>40</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F10" s="13">
+      <c r="F10" s="12">
         <f>SUMIF(Journal!$B$4:$B$203,A10,Journal!$D$4:$D$203)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="13">
         <f>'Tableau de bord'!$B$3+H10*7</f>
         <v>46391</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="10">
         <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="20"/>
-      <c r="B11" s="21" t="s">
+      <c r="A11" s="19"/>
+      <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="21">
         <f>SUM(C4:C10)</f>
         <v>275</v>
       </c>
-      <c r="D11" s="20"/>
-      <c r="E11" s="23">
+      <c r="D11" s="19"/>
+      <c r="E11" s="22">
         <f>SUMPRODUCT(C4:C10,E4:E10)/SUM(C4:C10)</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="22">
+        <v>0.12727272727272726</v>
+      </c>
+      <c r="F11" s="21">
         <f>SUM(F4:F10)</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
+        <v>5.2</v>
+      </c>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -1811,387 +1835,417 @@
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="3" max="3" width="55.33203125" customWidth="1"/>
     <col min="4" max="4" width="9" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="5" max="5" width="155.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="24"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="25"/>
+      <c r="A4" s="23">
+        <v>46209</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="25">
+        <v>2</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="27"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="28"/>
+      <c r="A5" s="26">
+        <v>46211</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="28">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="24"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="25"/>
+      <c r="A6" s="23">
+        <v>46220</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="25">
+        <v>1</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="27"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="28"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="27"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="24"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="25"/>
+      <c r="A8" s="23"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="24"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="27"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="28"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="27"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="24"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="25"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="24"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="27"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="28"/>
+      <c r="A11" s="26"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="27"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="24"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="25"/>
+      <c r="A12" s="23"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="24"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="27"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="28"/>
+      <c r="A13" s="26"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="27"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="24"/>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="25"/>
+      <c r="A14" s="23"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="24"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="27"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="28"/>
+      <c r="A15" s="26"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="27"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="24"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="25"/>
+      <c r="A16" s="23"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="24"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="27"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="28"/>
+      <c r="A17" s="26"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="27"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="24"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="25"/>
+      <c r="A18" s="23"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="24"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="27"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="28"/>
+      <c r="A19" s="26"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="27"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="24"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="25"/>
+      <c r="A20" s="23"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="24"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="27"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="28"/>
+      <c r="A21" s="26"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="27"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="24"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="25"/>
+      <c r="A22" s="23"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="24"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="27"/>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="28"/>
+      <c r="A23" s="26"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="27"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="24"/>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="25"/>
+      <c r="A24" s="23"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="24"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="27"/>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="28"/>
+      <c r="A25" s="26"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="27"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="24"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="25"/>
+      <c r="A26" s="23"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="24"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="27"/>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="28"/>
+      <c r="A27" s="26"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="27"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="24"/>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="25"/>
+      <c r="A28" s="23"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="24"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="27"/>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="28"/>
+      <c r="A29" s="26"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="27"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="24"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="25"/>
+      <c r="A30" s="23"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="24"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="27"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="28"/>
+      <c r="A31" s="26"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="27"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="24"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="25"/>
+      <c r="A32" s="23"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="24"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="27"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="28"/>
+      <c r="A33" s="26"/>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="27"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="24"/>
-      <c r="B34" s="25"/>
-      <c r="C34" s="25"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="25"/>
+      <c r="A34" s="23"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="24"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="27"/>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="29"/>
-      <c r="E35" s="28"/>
+      <c r="A35" s="26"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="27"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="24"/>
-      <c r="B36" s="25"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="25"/>
+      <c r="A36" s="23"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="24"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="27"/>
-      <c r="B37" s="28"/>
-      <c r="C37" s="28"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="28"/>
+      <c r="A37" s="26"/>
+      <c r="B37" s="27"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="27"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="24"/>
-      <c r="B38" s="25"/>
-      <c r="C38" s="25"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="25"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="25"/>
+      <c r="E38" s="24"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="27"/>
-      <c r="B39" s="28"/>
-      <c r="C39" s="28"/>
-      <c r="D39" s="29"/>
-      <c r="E39" s="28"/>
+      <c r="A39" s="26"/>
+      <c r="B39" s="27"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="27"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="24"/>
-      <c r="B40" s="25"/>
-      <c r="C40" s="25"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="25"/>
+      <c r="A40" s="23"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="25"/>
+      <c r="E40" s="24"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="27"/>
-      <c r="B41" s="28"/>
-      <c r="C41" s="28"/>
-      <c r="D41" s="29"/>
-      <c r="E41" s="28"/>
+      <c r="A41" s="26"/>
+      <c r="B41" s="27"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="27"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="24"/>
-      <c r="B42" s="25"/>
-      <c r="C42" s="25"/>
-      <c r="D42" s="26"/>
-      <c r="E42" s="25"/>
+      <c r="A42" s="23"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="24"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="27"/>
-      <c r="B43" s="28"/>
-      <c r="C43" s="28"/>
-      <c r="D43" s="29"/>
-      <c r="E43" s="28"/>
+      <c r="A43" s="26"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="27"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="24"/>
-      <c r="B44" s="25"/>
-      <c r="C44" s="25"/>
-      <c r="D44" s="26"/>
-      <c r="E44" s="25"/>
+      <c r="A44" s="23"/>
+      <c r="B44" s="24"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="25"/>
+      <c r="E44" s="24"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="27"/>
-      <c r="B45" s="28"/>
-      <c r="C45" s="28"/>
-      <c r="D45" s="29"/>
-      <c r="E45" s="28"/>
+      <c r="A45" s="26"/>
+      <c r="B45" s="27"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="27"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="24"/>
-      <c r="B46" s="25"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="26"/>
-      <c r="E46" s="25"/>
+      <c r="A46" s="23"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="24"/>
+      <c r="D46" s="25"/>
+      <c r="E46" s="24"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="27"/>
-      <c r="B47" s="28"/>
-      <c r="C47" s="28"/>
-      <c r="D47" s="29"/>
-      <c r="E47" s="28"/>
+      <c r="A47" s="26"/>
+      <c r="B47" s="27"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="27"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="24"/>
-      <c r="B48" s="25"/>
-      <c r="C48" s="25"/>
-      <c r="D48" s="26"/>
-      <c r="E48" s="25"/>
+      <c r="A48" s="23"/>
+      <c r="B48" s="24"/>
+      <c r="C48" s="24"/>
+      <c r="D48" s="25"/>
+      <c r="E48" s="24"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" s="27"/>
-      <c r="B49" s="28"/>
-      <c r="C49" s="28"/>
-      <c r="D49" s="29"/>
-      <c r="E49" s="28"/>
+      <c r="A49" s="26"/>
+      <c r="B49" s="27"/>
+      <c r="C49" s="27"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="27"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" s="24"/>
-      <c r="B50" s="25"/>
-      <c r="C50" s="25"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="25"/>
+      <c r="A50" s="23"/>
+      <c r="B50" s="24"/>
+      <c r="C50" s="24"/>
+      <c r="D50" s="25"/>
+      <c r="E50" s="24"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" s="27"/>
-      <c r="B51" s="28"/>
-      <c r="C51" s="28"/>
-      <c r="D51" s="29"/>
-      <c r="E51" s="28"/>
+      <c r="A51" s="26"/>
+      <c r="B51" s="27"/>
+      <c r="C51" s="27"/>
+      <c r="D51" s="28"/>
+      <c r="E51" s="27"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" s="24"/>
-      <c r="B52" s="25"/>
-      <c r="C52" s="25"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="25"/>
+      <c r="A52" s="23"/>
+      <c r="B52" s="24"/>
+      <c r="C52" s="24"/>
+      <c r="D52" s="25"/>
+      <c r="E52" s="24"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" s="27"/>
-      <c r="B53" s="28"/>
-      <c r="C53" s="28"/>
-      <c r="D53" s="29"/>
-      <c r="E53" s="28"/>
+      <c r="A53" s="26"/>
+      <c r="B53" s="27"/>
+      <c r="C53" s="27"/>
+      <c r="D53" s="28"/>
+      <c r="E53" s="27"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>